<commit_message>
Wertrechner Phase 2: Rechenkern, Berliner Modellschicht und Tests
- wertrechner/rechenkern.js: Sachwert- und allgemeines Ertragswertverfahren
  nach §§ 27-39 ImmoWertV als reine Rechenlogik ohne Abhängigkeiten; jeder
  Schritt mit Paragraf und ImmoWertA-Fundstelle protokolliert.
- wertrechner/berlin.js: setzt Besucherangaben und Adressdaten nach dem
  Berliner Modell um (NHK-Typ, RND-Tabellen, Sachwertfaktor- und
  Liegenschaftszins-Formeln, GFZ-Anpassung, Bewirtschaftungskosten,
  Gültigkeitsprüfungen, Wertspanne).
- tests/: Referenzfall A (Sachwert 692.000 €, Ertragswert 687.000 €) exakt;
  Randfälle; Tabellenwerte des Gutachterausschusses nachgerechnet.
- Entscheidungen zu Rundung, GFZ außerhalb der Tabellen, Wohnlage sehr gut,
  Gültigkeitsbereichen, Wertspanne und BGF-Ableitung in MODELL-BERLIN.md.
</commit_message>
<xml_diff>
--- a/daten/marktdaten.xlsx
+++ b/daten/marktdaten.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -931,45 +931,45 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>bgf_faktor_unterkellert</t>
+          <t>wohnflaeche_anteil_vollgeschoss</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1.55</v>
+        <v>0.8</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Faktor</t>
+          <t>Anteil</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Schätzung BGF = Wohnfläche × Faktor, wenn nur die Wohnfläche bekannt ist (unterkellert)</t>
+          <t>Schätzung der BGF aus der Wohnfläche: Wohnfläche eines Vollgeschosses im Verhältnis zur Grundfläche nach Außenmaßen</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Annahme BIB – bitte prüfen (MODELL-BERLIN.md Abschnitt 7)</t>
+          <t>Annahme BIB – bitte prüfen (MODELL-BERLIN.md Abschnitt 7); Erfahrungswert 70–80 % (Wandanteile, Treppe)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>bgf_faktor_nicht_unterkellert</t>
+          <t>wohnflaeche_anteil_dachgeschoss</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1.3</v>
+        <v>0.55</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Faktor</t>
+          <t>Anteil</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Schätzung BGF = Wohnfläche × Faktor (nicht unterkellert)</t>
+          <t>Schätzung der BGF aus der Wohnfläche: Wohnfläche eines voll ausgebauten Dachgeschosses im Verhältnis zur Grundfläche</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -981,45 +981,45 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ertragswert_mindest_mieteinheiten</t>
+          <t>bgf_anteil_dachgeschoss</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>4</v>
+        <v>0.8</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Anzahl</t>
+          <t>Anteil</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Liegenschaftszinssätze gelten ab vier Mieteinheiten</t>
+          <t>Anrechenbare Dachgeschossfläche (nutzbar, Giebelhöhe &gt; 1,50 m) im Verhältnis zur Grundfläche – für die Ableitung der BGF aus Grundfläche oder Wohnfläche</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Liegenschaftszinssätze 2025 (Stand 24.10.2025) S. 1</t>
+          <t>Annahme BIB – bitte prüfen (MODELL-BERLIN.md Abschnitt 7); BGF-Regeln Sachwertfaktoren 2025 (Stand 04.02.2026) S. 3</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ertragswert_max_gewerbeanteil_prozent</t>
+          <t>ertragswert_mindest_mieteinheiten</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>Anzahl</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Gewerblicher Anteil am Nettojahresrohertrag höchstens</t>
+          <t>Liegenschaftszinssätze gelten ab vier Mieteinheiten</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1031,64 +1031,62 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ertragswert_baujahr_min</t>
+          <t>ertragswert_max_gewerbeanteil_prozent</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1865</v>
+        <v>80</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Jahr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Jüngstes Baujahr in der Ableitung</t>
+          <t>Gewerblicher Anteil am Nettojahresrohertrag höchstens</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Liegenschaftszinssätze 2025 (Stand 24.10.2025) S. 2</t>
+          <t>Liegenschaftszinssätze 2025 (Stand 24.10.2025) S. 1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>gfz_w_formel</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>K(GFZ) = (−25,191 + 311,62·GFZ − 24,879·GFZ²) / 498,533; gültig 0,8–5,0; auf GFZ 2,0 = 1,0000 basiert</t>
-        </is>
+          <t>ertragswert_baujahr_min</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1865</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Jahr</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Hintergrund der Tabelle Wohn-04; der Rechner nutzt die Tabelle mit linearer Zwischenwertbildung</t>
+          <t>Jüngstes Baujahr in der Ableitung</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>GFZ-Umrechnungskoeffizienten Wohnbauland 2004 (Stand 12.10.2022) S. 2</t>
+          <t>Liegenschaftszinssätze 2025 (Stand 24.10.2025) S. 2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>gfz_d_formel</t>
+          <t>gfz_w_formel</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>K(GFZ) = 0,2047·GFZ + 0,181; gültig 2,0–7,0; auf GFZ 4,0 = 1,0000 basiert</t>
+          <t>K(GFZ) = (−25,191 + 311,62·GFZ − 24,879·GFZ²) / 498,533; gültig 0,8–5,0; auf GFZ 2,0 = 1,0000 basiert</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1098,37 +1096,64 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Hintergrund der Tabelle Dienst-04</t>
+          <t>Hintergrund der Tabelle Wohn-04; der Rechner nutzt die Tabelle mit linearer Zwischenwertbildung</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>GFZ-Umrechnungskoeffizienten Dienstleistung 2004 (Stand 12.10.2022) S. 2</t>
+          <t>GFZ-Umrechnungskoeffizienten Wohnbauland 2004 (Stand 12.10.2022) S. 2</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>gfz_d_formel</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>K(GFZ) = 0,2047·GFZ + 0,181; gültig 2,0–7,0; auf GFZ 4,0 = 1,0000 basiert</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Hintergrund der Tabelle Dienst-04</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>GFZ-Umrechnungskoeffizienten Dienstleistung 2004 (Stand 12.10.2022) S. 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>wohnlagen_datensatz</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>Wohnlagen nach Adressen zum Berliner Mietspiegel 2024</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>Quelle der automatischen Wohnlage je Adresse</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>Geoportal Berlin, WFS wohnlagenadr2024</t>
         </is>

</xml_diff>